<commit_message>
Update SmartPay Dashboard and project files
</commit_message>
<xml_diff>
--- a/data/IS Issues.xlsx
+++ b/data/IS Issues.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1440" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1440" uniqueCount="257">
   <si>
     <t>Severity</t>
   </si>
@@ -822,6 +822,9 @@
   </si>
   <si>
     <t>Fixation in Progress</t>
+  </si>
+  <si>
+    <t>Under Revalidation</t>
   </si>
 </sst>
 </file>
@@ -4561,7 +4564,7 @@
         <v>249</v>
       </c>
       <c r="D189" s="7" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E189" s="8" t="s">
         <v>253</v>

</xml_diff>